<commit_message>
rebuild nigeria content as coding units matching kibe reference schema
</commit_message>
<xml_diff>
--- a/Content Analysis - Nigeria/_summary.xlsx
+++ b/Content Analysis - Nigeria/_summary.xlsx
@@ -14,15 +14,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="16">
-  <si>
-    <t>creator</t>
-  </si>
-  <si>
-    <t>orientation</t>
-  </si>
-  <si>
-    <t>pieces</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
+  <si>
+    <t>influencer</t>
+  </si>
+  <si>
+    <t>units</t>
   </si>
   <si>
     <t>path</t>
@@ -43,25 +40,19 @@
     <t>Wizarab</t>
   </si>
   <si>
-    <t>Regressive</t>
-  </si>
-  <si>
-    <t>Progressive</t>
-  </si>
-  <si>
-    <t>Content Analysis - Nigeria/Agba John Doe/Agba John Doe_content.xlsx</t>
-  </si>
-  <si>
-    <t>Content Analysis - Nigeria/Banky Wellington/Banky Wellington_content.xlsx</t>
-  </si>
-  <si>
-    <t>Content Analysis - Nigeria/Deyemi Okanlawon/Deyemi Okanlawon_content.xlsx</t>
-  </si>
-  <si>
-    <t>Content Analysis - Nigeria/Shola/Shola_content.xlsx</t>
-  </si>
-  <si>
-    <t>Content Analysis - Nigeria/Wizarab/Wizarab_content.xlsx</t>
+    <t>Content Analysis - Nigeria/Agba John Doe/Agba John Doe_Coding_Units.xlsx</t>
+  </si>
+  <si>
+    <t>Content Analysis - Nigeria/Banky Wellington/Banky Wellington_Coding_Units.xlsx</t>
+  </si>
+  <si>
+    <t>Content Analysis - Nigeria/Deyemi Okanlawon/Deyemi Okanlawon_Coding_Units.xlsx</t>
+  </si>
+  <si>
+    <t>Content Analysis - Nigeria/Shola/Shola_Coding_Units.xlsx</t>
+  </si>
+  <si>
+    <t>Content Analysis - Nigeria/Wizarab/Wizarab_Coding_Units.xlsx</t>
   </si>
 </sst>
 </file>
@@ -419,10 +410,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:4">
+    <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -432,78 +423,60 @@
       <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="2" spans="1:4">
-      <c r="A2" t="s">
+      <c r="B2">
+        <v>5</v>
+      </c>
+      <c r="C2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
+      <c r="A3" t="s">
         <v>4</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B3">
+        <v>40</v>
+      </c>
+      <c r="C3" t="s">
         <v>9</v>
       </c>
-      <c r="C2">
+    </row>
+    <row r="4" spans="1:3">
+      <c r="A4" t="s">
         <v>5</v>
       </c>
-      <c r="D2" t="s">
+      <c r="B4">
+        <v>4</v>
+      </c>
+      <c r="C4" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3">
+      <c r="A5" t="s">
+        <v>6</v>
+      </c>
+      <c r="B5">
+        <v>5</v>
+      </c>
+      <c r="C5" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:4">
-      <c r="A3" t="s">
+    <row r="6" spans="1:3">
+      <c r="A6" t="s">
+        <v>7</v>
+      </c>
+      <c r="B6">
         <v>5</v>
       </c>
-      <c r="B3" t="s">
-        <v>10</v>
-      </c>
-      <c r="C3">
-        <v>40</v>
-      </c>
-      <c r="D3" t="s">
+      <c r="C6" t="s">
         <v>12</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4">
-      <c r="A4" t="s">
-        <v>6</v>
-      </c>
-      <c r="B4" t="s">
-        <v>10</v>
-      </c>
-      <c r="C4">
-        <v>4</v>
-      </c>
-      <c r="D4" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4">
-      <c r="A5" t="s">
-        <v>7</v>
-      </c>
-      <c r="B5" t="s">
-        <v>9</v>
-      </c>
-      <c r="C5">
-        <v>5</v>
-      </c>
-      <c r="D5" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4">
-      <c r="A6" t="s">
-        <v>8</v>
-      </c>
-      <c r="B6" t="s">
-        <v>9</v>
-      </c>
-      <c r="C6">
-        <v>5</v>
-      </c>
-      <c r="D6" t="s">
-        <v>15</v>
       </c>
     </row>
   </sheetData>

</xml_diff>